<commit_message>
Cambios en la estructuracion de los eventos
</commit_message>
<xml_diff>
--- a/servicios.xlsx
+++ b/servicios.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Desktop\DOO\DOO\Barberia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/120f6d501c463b80/Escritorio/leo/Doo/Barberia proyecto/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AB46960-CA2B-4571-925B-D430D14FB839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{3AB46960-CA2B-4571-925B-D430D14FB839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{518DDA80-B1AD-47BE-BE23-473973EC73CB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Responsablidades" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="83">
   <si>
     <t>Servicio</t>
   </si>
@@ -92,9 +92,6 @@
     <t>Modificar las políticas</t>
   </si>
   <si>
-    <t>Ajustar precio de un servicio</t>
-  </si>
-  <si>
     <t>Ver la regla definida</t>
   </si>
   <si>
@@ -128,27 +125,12 @@
     <t>Desactivar horario de barberia</t>
   </si>
   <si>
-    <t>Editar mi contacto</t>
-  </si>
-  <si>
     <t>Editar tiempos de anticipación de citas</t>
   </si>
   <si>
-    <t>Consultar la información de un cliente</t>
-  </si>
-  <si>
-    <t>Consultar la información de un barbero</t>
-  </si>
-  <si>
-    <t>Ver si estoy vetado</t>
-  </si>
-  <si>
     <t>Dejar de trabajar en la barbería</t>
   </si>
   <si>
-    <t>Ver cuántos descuentos tengo para mis futuras citas</t>
-  </si>
-  <si>
     <t>HorarioBarbero</t>
   </si>
   <si>
@@ -170,9 +152,6 @@
     <t>Desactivar horario de trabajo</t>
   </si>
   <si>
-    <t>Ver mis servicios</t>
-  </si>
-  <si>
     <t>Ver horarios de trabajo de un barbero</t>
   </si>
   <si>
@@ -257,22 +236,52 @@
     <t>Definir un bloque de no disponible</t>
   </si>
   <si>
-    <t>Borrar un bloqueo</t>
-  </si>
-  <si>
-    <t>Ver bloqueos en un rango de fechas</t>
-  </si>
-  <si>
     <t>Ver bloqueos de una fecha</t>
   </si>
   <si>
-    <t>Ajustar el nombre de un servicio</t>
-  </si>
-  <si>
-    <t>Ajustar la descripcion de un servicio</t>
-  </si>
-  <si>
     <t>Ver descripción de un estado</t>
+  </si>
+  <si>
+    <t>Editar un servicio</t>
+  </si>
+  <si>
+    <t>Editar contacto</t>
+  </si>
+  <si>
+    <t>Cliente, Barbero</t>
+  </si>
+  <si>
+    <t>Ver datos de un barbero</t>
+  </si>
+  <si>
+    <t>Ver mis tiempos de anticipación para las citas</t>
+  </si>
+  <si>
+    <t>Ver datos de un cliente</t>
+  </si>
+  <si>
+    <t>Ver estado de vetado</t>
+  </si>
+  <si>
+    <t>Ver cantidad de descuentos para las citas</t>
+  </si>
+  <si>
+    <t>Ver cantidad de multas sin pagar</t>
+  </si>
+  <si>
+    <t>Ver tiempos de anticipacion para las citas</t>
+  </si>
+  <si>
+    <t>Ver servicios elegidos</t>
+  </si>
+  <si>
+    <t>Editar un bloqueo</t>
+  </si>
+  <si>
+    <t>Eliminar un bloqueo</t>
+  </si>
+  <si>
+    <t>Ver bloqueo de una fecha y hora</t>
   </si>
 </sst>
 </file>
@@ -374,7 +383,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -395,6 +404,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -410,6 +423,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -675,23 +692,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:R60"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B2:U61"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="41.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" customWidth="1"/>
-    <col min="5" max="5" width="42.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.44140625" customWidth="1"/>
-    <col min="8" max="8" width="35.44140625" customWidth="1"/>
-    <col min="9" max="9" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="32.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.88671875" customWidth="1"/>
-    <col min="14" max="14" width="30.5546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.44140625" customWidth="1"/>
-    <col min="17" max="17" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
+    <col min="5" max="5" width="42.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" customWidth="1"/>
+    <col min="8" max="8" width="35.42578125" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.85546875" customWidth="1"/>
+    <col min="14" max="14" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.42578125" customWidth="1"/>
+    <col min="17" max="17" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="33.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
         <v>0</v>
       </c>
@@ -716,8 +734,12 @@
         <v>5</v>
       </c>
       <c r="R2" s="11"/>
-    </row>
-    <row r="3" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="T2" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="U2" s="11"/>
+    </row>
+    <row r="3" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
@@ -754,8 +776,14 @@
       <c r="R3" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="2:18" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="T3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="2:21" ht="30" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>8</v>
       </c>
@@ -792,10 +820,16 @@
       <c r="R4" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="2:18" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="T4" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="2:21" ht="30" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>9</v>
@@ -803,7 +837,7 @@
       <c r="E5" s="8"/>
       <c r="F5" s="9"/>
       <c r="H5" s="4" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>13</v>
@@ -818,16 +852,22 @@
       </c>
       <c r="Q5" s="9"/>
       <c r="R5" s="9"/>
-    </row>
-    <row r="6" spans="2:18" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="T5" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="U5" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="2:21" ht="45" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>9</v>
+        <v>20</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>9</v>
@@ -835,15 +875,21 @@
       <c r="K6" s="6"/>
       <c r="L6" s="6"/>
       <c r="N6" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O6" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="7" spans="2:18" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="T6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="U6" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="2:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>9</v>
@@ -853,492 +899,477 @@
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
       <c r="R7" s="5"/>
-    </row>
-    <row r="8" spans="2:18" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B8" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>13</v>
-      </c>
+      <c r="T7" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="U7" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="2:21" x14ac:dyDescent="0.25">
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
       <c r="K8" s="6"/>
       <c r="L8" s="6"/>
-    </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B9" s="3" t="s">
+      <c r="T8" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="U8" s="13" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B12" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C12" s="11"/>
+      <c r="E12" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" s="11"/>
+      <c r="H12" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="I12" s="11"/>
+    </row>
+    <row r="13" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="2:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B13" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="11"/>
-      <c r="E13" s="10" t="s">
+      <c r="E14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I14" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F13" s="11"/>
-      <c r="H13" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="I13" s="11"/>
-    </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B14" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B15" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="3" t="s">
+    </row>
+    <row r="15" spans="2:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E15" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="2:18" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>13</v>
-      </c>
       <c r="E16" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>31</v>
+        <v>74</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B17" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>9</v>
-      </c>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="E17" s="4" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>24</v>
+        <v>71</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>33</v>
+        <v>75</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:9" ht="30" x14ac:dyDescent="0.25">
       <c r="E18" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E19" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E20" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" s="11"/>
+      <c r="E24" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F24" s="11"/>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B26" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="F18" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H18" s="4" t="s">
+      <c r="C26" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="I18" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="E19" s="4" t="s">
+      <c r="F26" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B27" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="C27" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B28" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B29" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C29" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="H19" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="I19" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B23" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C23" s="11"/>
-      <c r="E23" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="F23" s="11"/>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B24" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B25" s="3" t="s">
+      <c r="E29" s="3" t="s">
         <v>40</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B26" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B27" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B28" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="E29" s="3" t="s">
-        <v>48</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B33" s="10" t="s">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E30" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B34" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C34" s="11"/>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B35" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B36" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B39" s="6"/>
+      <c r="C39" s="6"/>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B42" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C42" s="11"/>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B43" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B44" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C33" s="11"/>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B34" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B35" s="4" t="s">
+      <c r="C44" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B45" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C45" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B46" s="4" t="s">
         <v>51</v>
-      </c>
-    </row>
-    <row r="36" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="37" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B38" s="6"/>
-      <c r="C38" s="6"/>
-    </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B41" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="C41" s="11"/>
-      <c r="E41" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="F41" s="11"/>
-    </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B42" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B43" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F43" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B44" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="F44" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B45" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E45" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="F45" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B46" s="4" t="s">
-        <v>59</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E46" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F46" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B47" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B48" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E48" s="8"/>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B49" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B50" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B51" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B52" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B53" s="5"/>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B54" s="5"/>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B56" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C56" s="11"/>
+      <c r="E56" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="F56" s="11"/>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B57" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B58" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E47" s="8"/>
-    </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B48" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="49" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B49" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B50" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B51" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B52" s="5"/>
-    </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B53" s="5"/>
-    </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B55" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="C55" s="11"/>
-      <c r="E55" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="F55" s="11"/>
-    </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B56" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B57" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E57" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="58" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B58" s="4" t="s">
-        <v>72</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>11</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B59" s="8"/>
-      <c r="C59" s="8"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B59" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="E59" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F59" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="F59" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G59" s="6"/>
-    </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B60" s="8"/>
       <c r="C60" s="8"/>
-      <c r="E60" s="8"/>
-      <c r="F60" s="8"/>
+      <c r="E60" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G60" s="6"/>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B61" s="8"/>
+      <c r="C61" s="8"/>
+      <c r="E61" s="8"/>
+      <c r="F61" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="E55:F55"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="E56:F56"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="E24:F24"/>
     <mergeCell ref="Q2:R2"/>
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="K2:L2"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="H12:I12"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="H2:I2"/>
   </mergeCells>

</xml_diff>

<commit_message>
ELiminacion y cambios de los archivos
</commit_message>
<xml_diff>
--- a/servicios.xlsx
+++ b/servicios.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/120f6d501c463b80/Escritorio/leo/Doo/Barberia proyecto/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Desktop\DOO\DOO\Barberia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{3AB46960-CA2B-4571-925B-D430D14FB839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{518DDA80-B1AD-47BE-BE23-473973EC73CB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6B90A86-FEF4-4074-99A8-56667ECFA95C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Responsablidades" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="84">
   <si>
     <t>Servicio</t>
   </si>
@@ -281,7 +281,10 @@
     <t>Eliminar un bloqueo</t>
   </si>
   <si>
-    <t>Ver bloqueo de una fecha y hora</t>
+    <t>Ver bloqueo de una fecha y hora de inicio</t>
+  </si>
+  <si>
+    <t>Añadir prefijo celular para los contactos</t>
   </si>
 </sst>
 </file>
@@ -383,7 +386,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -404,10 +407,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -423,10 +422,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -693,23 +688,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:U61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="41.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" customWidth="1"/>
-    <col min="5" max="5" width="42.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" customWidth="1"/>
-    <col min="8" max="8" width="35.42578125" customWidth="1"/>
-    <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="32.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.85546875" customWidth="1"/>
-    <col min="14" max="14" width="30.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.42578125" customWidth="1"/>
-    <col min="17" max="17" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.44140625" customWidth="1"/>
+    <col min="5" max="5" width="42.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.44140625" customWidth="1"/>
+    <col min="8" max="8" width="35.44140625" customWidth="1"/>
+    <col min="9" max="9" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.88671875" customWidth="1"/>
+    <col min="14" max="14" width="30.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.44140625" customWidth="1"/>
+    <col min="17" max="17" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="33.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B2" s="10" t="s">
         <v>0</v>
       </c>
@@ -739,7 +734,7 @@
       </c>
       <c r="U2" s="11"/>
     </row>
-    <row r="3" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
@@ -783,7 +778,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
         <v>8</v>
       </c>
@@ -827,15 +822,19 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="2:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>69</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="8"/>
-      <c r="F5" s="9"/>
+      <c r="E5" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="H5" s="4" t="s">
         <v>68</v>
       </c>
@@ -859,7 +858,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="2:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B6" s="4" t="s">
         <v>20</v>
       </c>
@@ -887,7 +886,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="2:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:21" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>21</v>
       </c>
@@ -899,26 +898,26 @@
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
       <c r="R7" s="5"/>
-      <c r="T7" s="3" t="s">
+      <c r="T7" s="4" t="s">
         <v>82</v>
       </c>
       <c r="U7" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:21" x14ac:dyDescent="0.3">
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
       <c r="K8" s="6"/>
       <c r="L8" s="6"/>
-      <c r="T8" s="13" t="s">
+      <c r="T8" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="U8" s="13" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="U8" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B12" s="10" t="s">
         <v>22</v>
       </c>
@@ -932,7 +931,7 @@
       </c>
       <c r="I12" s="11"/>
     </row>
-    <row r="13" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>6</v>
       </c>
@@ -952,7 +951,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>25</v>
       </c>
@@ -972,7 +971,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="2:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:21" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="4" t="s">
         <v>28</v>
       </c>
@@ -992,7 +991,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>29</v>
       </c>
@@ -1012,7 +1011,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
       <c r="E17" s="4" t="s">
         <v>72</v>
       </c>
@@ -1026,7 +1025,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
       <c r="E18" s="4" t="s">
         <v>31</v>
       </c>
@@ -1040,29 +1039,29 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="E19" s="12" t="s">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="E19" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="F19" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="H19" s="12" t="s">
+      <c r="F19" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H19" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="I19" s="12" t="s">
+      <c r="I19" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="E20" s="12" t="s">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="E20" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="F20" s="12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="F20" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B24" s="10" t="s">
         <v>32</v>
       </c>
@@ -1072,7 +1071,7 @@
       </c>
       <c r="F24" s="11"/>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B25" s="1" t="s">
         <v>6</v>
       </c>
@@ -1086,7 +1085,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
         <v>34</v>
       </c>
@@ -1100,7 +1099,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B27" s="4" t="s">
         <v>36</v>
       </c>
@@ -1114,7 +1113,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B28" s="3" t="s">
         <v>38</v>
       </c>
@@ -1128,7 +1127,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>39</v>
       </c>
@@ -1142,7 +1141,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
       <c r="E30" s="3" t="s">
         <v>41</v>
       </c>
@@ -1150,13 +1149,13 @@
         <v>23</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B34" s="10" t="s">
         <v>42</v>
       </c>
       <c r="C34" s="11"/>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B35" s="1" t="s">
         <v>6</v>
       </c>
@@ -1164,7 +1163,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B36" s="4" t="s">
         <v>43</v>
       </c>
@@ -1172,7 +1171,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="4" t="s">
         <v>45</v>
       </c>
@@ -1180,7 +1179,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="4" t="s">
         <v>46</v>
       </c>
@@ -1188,17 +1187,17 @@
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
     </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B42" s="10" t="s">
         <v>47</v>
       </c>
       <c r="C42" s="11"/>
     </row>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B43" s="1" t="s">
         <v>6</v>
       </c>
@@ -1206,7 +1205,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B44" s="4" t="s">
         <v>49</v>
       </c>
@@ -1214,7 +1213,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B45" s="4" t="s">
         <v>50</v>
       </c>
@@ -1222,7 +1221,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B46" s="4" t="s">
         <v>51</v>
       </c>
@@ -1230,7 +1229,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B47" s="4" t="s">
         <v>52</v>
       </c>
@@ -1238,7 +1237,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B48" s="4" t="s">
         <v>53</v>
       </c>
@@ -1247,7 +1246,7 @@
       </c>
       <c r="E48" s="8"/>
     </row>
-    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B49" s="4" t="s">
         <v>54</v>
       </c>
@@ -1255,7 +1254,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B50" s="4" t="s">
         <v>55</v>
       </c>
@@ -1263,7 +1262,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B51" s="4" t="s">
         <v>56</v>
       </c>
@@ -1271,7 +1270,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B52" s="4" t="s">
         <v>57</v>
       </c>
@@ -1279,13 +1278,13 @@
         <v>44</v>
       </c>
     </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B53" s="5"/>
     </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B54" s="5"/>
     </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B56" s="10" t="s">
         <v>58</v>
       </c>
@@ -1295,7 +1294,7 @@
       </c>
       <c r="F56" s="11"/>
     </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B57" s="1" t="s">
         <v>6</v>
       </c>
@@ -1309,7 +1308,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B58" s="3" t="s">
         <v>60</v>
       </c>
@@ -1323,7 +1322,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B59" s="4" t="s">
         <v>65</v>
       </c>
@@ -1337,7 +1336,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B60" s="8"/>
       <c r="C60" s="8"/>
       <c r="E60" s="4" t="s">
@@ -1348,7 +1347,7 @@
       </c>
       <c r="G60" s="6"/>
     </row>
-    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B61" s="8"/>
       <c r="C61" s="8"/>
       <c r="E61" s="8"/>

</xml_diff>